<commit_message>
Add Riyadh sales before 30-7-2025 to sales workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/إجمالي_مبيعات_المناديب_30-7-2025_إلى_31-7-2026.xlsx
+++ b/إجمالي_مبيعات_المناديب_30-7-2025_إلى_31-7-2026.xlsx
@@ -10,16 +10,17 @@
     <sheet name="الملخص" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="الحركة المدمجة" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="ملخص شهري حسب المندوب" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="مبيعات عصمت" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="مبيعات عماد" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="مبيعات أبو خالد" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="أبو خالد - تفصيل البنود" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="مبيعات قبل 30.7.2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="مبيعات عصمت" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="مبيعات عماد" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="مبيعات أبو خالد" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="أبو خالد - تفصيل البنود" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'الحركة المدمجة'!$A$1:$J$360</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'مبيعات عصمت'!$A$1:$I$255</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'مبيعات عماد'!$A$1:$I$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'مبيعات أبو خالد'!$A$1:$I$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'مبيعات عصمت'!$A$1:$I$255</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'مبيعات عماد'!$A$1:$I$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'مبيعات أبو خالد'!$A$1:$I$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,11 +28,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +49,10 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="10">
@@ -125,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -176,6 +180,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -541,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -563,11 +568,10 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>الفترة كاملة: من 30-7-2025 إلى 31-7-2026 – دمج شيت المبيعات (عقود الجملة من 30-7-2025 حتى 3-6-2026) مع النظام الجديد المسمى برقم السيارة (شهري 6 و7 لسنة 2026: سيارة 1219 = عصمت، سيارة 3010 = عماد)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>الفترة كاملة: من 1-10-2024 إلى 31-7-2026 – مبيعات ما قبل 30-7-2025 (إجمالي شهري غير موزع على المناديب) + شيت المبيعات (عقود الجملة من 30-7-2025 حتى 3-6-2026) + النظام الجديد برقم السيارة (شهري 6 و7 لسنة 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -702,121 +706,140 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>الإجمالي</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>SUM(B5:B7)</f>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات قبل 30.7.2025 (1-10-2024 إلى 30-6-2025) – غير موزعة على المناديب</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="4">
+        <f>'مبيعات قبل 30.7.2025'!C12</f>
         <v/>
       </c>
-      <c r="C8" s="6">
-        <f>SUM(C5:C7)</f>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>الإجمالي الكلي (1-10-2024 إلى 31-7-2026)</t>
+        </is>
+      </c>
+      <c r="B9" s="6">
+        <f>SUM(B5:B8)</f>
         <v/>
       </c>
-      <c r="D8" s="6">
-        <f>SUM(D5:D7)</f>
+      <c r="C9" s="6">
+        <f>SUM(C5:C8)</f>
         <v/>
       </c>
-      <c r="E8" s="6">
-        <f>SUM(E5:E7)</f>
+      <c r="D9" s="6">
+        <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="F8" s="6">
-        <f>SUM(F5:F7)</f>
+      <c r="E9" s="6">
+        <f>SUM(E5:E8)</f>
         <v/>
       </c>
-      <c r="G8" s="5" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr"/>
+      <c r="F9" s="6">
+        <f>SUM(F5:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>ملاحظات المراجعة (كل الأرقام بالقيمة الإجمالية كما هي بالمستندات):</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>1) عصمت (WHT): شيت المحاسب مكتوب "من 9-10-2025" لكنه أدرج عقوداً من يوليو–سبتمبر، وأسقط 4 عقود من 1 إلى 8 أكتوبر (WHT-2348/2358/2378/2408 = 21,087.50) فتمت إضافتها.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>2) عصمت: عقدان WHT-2756 و WHT-2758 (16,810.00) موجودان في سجل العقود فقط، بدون فاتورة مبدئية ولا قيد في الكشف – تمت إضافتهما.</t>
+          <t>1) عصمت (WHT): شيت المحاسب مكتوب "من 9-10-2025" لكنه أدرج عقوداً من يوليو–سبتمبر، وأسقط 4 عقود من 1 إلى 8 أكتوبر (WHT-2348/2358/2378/2408 = 21,087.50) فتمت إضافتها.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>3) عصمت: 3 عقود مكررة الرقم في شيت المحاسب (WHT-3786 و WHT-4052 و WHT-4234) – القيم صحيحة والأرقام الصحيحة WHT-3804 و WHT-4062 و WHT-4243.</t>
+          <t>2) عصمت: عقدان WHT-2756 و WHT-2758 (16,810.00) موجودان في سجل العقود فقط، بدون فاتورة مبدئية ولا قيد في الكشف – تمت إضافتهما.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>4) العقدان WHT-1908 (16,658.75) و WHK-1909 (11,570.00) بتاريخ 30-7-2025 – بداية الفترة.</t>
+          <t>3) عصمت: 3 عقود مكررة الرقم في شيت المحاسب (WHT-3786 و WHT-4052 و WHT-4234) – القيم صحيحة والأرقام الصحيحة WHT-3804 و WHT-4062 و WHT-4243.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>5) أبو خالد (WHK): عقد عرعر WHK-2364 أُدرج بالقيمة الكاملة 440,000 بناءً على طلبك، علماً بأن المسجل بكشف الحساب 367,803.75 (الفرق 72,196.25 بدون قيد بالكشف).</t>
+          <t>4) العقدان WHT-1908 (16,658.75) و WHK-1909 (11,570.00) بتاريخ 30-7-2025 – بداية الفترة.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>6) أبو خالد: العقد WHK-3400 (505.00 – فاتورة 103) سقط من شيت المحاسب فتمت إضافته.</t>
+          <t>5) أبو خالد (WHK): عقد عرعر WHK-2364 أُدرج بالقيمة الكاملة 440,000 بناءً على طلبك، علماً بأن المسجل بكشف الحساب 367,803.75 (الفرق 72,196.25 بدون قيد بالكشف).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>7) عماد (WHE): الشيت مطابق تماماً للفواتير المبدئية وسجل العقود (45 عقد).</t>
+          <t>6) أبو خالد: العقد WHK-3400 (505.00 – فاتورة 103) سقط من شيت المحاسب فتمت إضافته.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>8) مبيعات النظام الجديد (برقم السيارة) مدمجة في صفحة كل مندوب: السيارة 1219 = عصمت، والسيارة 3010 = عماد. المحاسب لم يخصم 3 فواتير مرتجعة بالكامل لسيارة 1219 (4,123.90). شيت المرتجعات فيه صفّان مكرران (WS-RET-0002 و 0003).</t>
+          <t>7) عماد (WHE): الشيت مطابق تماماً للفواتير المبدئية وسجل العقود (45 عقد).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
+          <t>8) مبيعات النظام الجديد (برقم السيارة) مدمجة في صفحة كل مندوب: السيارة 1219 = عصمت، والسيارة 3010 = عماد. المحاسب لم يخصم 3 فواتير مرتجعة بالكامل لسيارة 1219 (4,123.90). شيت المرتجعات فيه صفّان مكرران (WS-RET-0002 و 0003).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
           <t>9) بعض التواريخ في ملفات المحاسب مقلوبة (يوم/شهر) مثل 2026-11-07 وهي 7-11 أي 11 يوليو – تم تصحيحها.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A9:G9"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13696,7 +13719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13740,380 +13763,524 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>أكتوبر 2024</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="n"/>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="11" t="n">
+        <v>103500</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>نوفمبر 2024</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="11" t="n">
+        <v>137450</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>ديسمبر 2024</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="11" t="n">
+        <v>95230</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>يناير 2025</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="11" t="n">
+        <v>55300</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>فبراير 2025</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="11" t="n">
+        <v>35920</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>مارس 2025</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="11" t="n">
+        <v>15100</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>إبريل 2025</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="11" t="n">
+        <v>90160</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>مايو 2025</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="11" t="n">
+        <v>50310</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>يونيه 2025</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="11" t="n">
+        <v>27718</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>07-2025</t>
         </is>
       </c>
-      <c r="B2" s="4">
+      <c r="B11" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,8,1))</f>
         <v/>
       </c>
-      <c r="C2" s="4">
+      <c r="C11" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,8,1))</f>
         <v/>
       </c>
-      <c r="D2" s="4">
+      <c r="D11" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,8,1))</f>
         <v/>
       </c>
-      <c r="E2" s="4">
+      <c r="E11" s="4">
         <f>SUM(B2:D2)</f>
         <v/>
       </c>
-      <c r="F2" s="4">
+      <c r="F11" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,8,1))</f>
         <v/>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>08-2025</t>
         </is>
       </c>
-      <c r="B3" s="4">
+      <c r="B12" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,8,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,9,1))</f>
         <v/>
       </c>
-      <c r="C3" s="4">
+      <c r="C12" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,8,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,9,1))</f>
         <v/>
       </c>
-      <c r="D3" s="4">
+      <c r="D12" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,8,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,9,1))</f>
         <v/>
       </c>
-      <c r="E3" s="4">
+      <c r="E12" s="4">
         <f>SUM(B3:D3)</f>
         <v/>
       </c>
-      <c r="F3" s="4">
+      <c r="F12" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,8,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,9,1))</f>
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>09-2025</t>
         </is>
       </c>
-      <c r="B4" s="4">
+      <c r="B13" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,9,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,10,1))</f>
         <v/>
       </c>
-      <c r="C4" s="4">
+      <c r="C13" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,9,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,10,1))</f>
         <v/>
       </c>
-      <c r="D4" s="4">
+      <c r="D13" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,9,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,10,1))</f>
         <v/>
       </c>
-      <c r="E4" s="4">
+      <c r="E13" s="4">
         <f>SUM(B4:D4)</f>
         <v/>
       </c>
-      <c r="F4" s="4">
+      <c r="F13" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,9,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,10,1))</f>
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>10-2025</t>
         </is>
       </c>
-      <c r="B5" s="4">
+      <c r="B14" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,10,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,11,1))</f>
         <v/>
       </c>
-      <c r="C5" s="4">
+      <c r="C14" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,10,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,11,1))</f>
         <v/>
       </c>
-      <c r="D5" s="4">
+      <c r="D14" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,10,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,11,1))</f>
         <v/>
       </c>
-      <c r="E5" s="4">
+      <c r="E14" s="4">
         <f>SUM(B5:D5)</f>
         <v/>
       </c>
-      <c r="F5" s="4">
+      <c r="F14" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,10,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,11,1))</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>11-2025</t>
         </is>
       </c>
-      <c r="B6" s="4">
+      <c r="B15" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,11,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,12,1))</f>
         <v/>
       </c>
-      <c r="C6" s="4">
+      <c r="C15" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,11,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,12,1))</f>
         <v/>
       </c>
-      <c r="D6" s="4">
+      <c r="D15" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,11,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,12,1))</f>
         <v/>
       </c>
-      <c r="E6" s="4">
+      <c r="E15" s="4">
         <f>SUM(B6:D6)</f>
         <v/>
       </c>
-      <c r="F6" s="4">
+      <c r="F15" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,11,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2025,12,1))</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>12-2025</t>
         </is>
       </c>
-      <c r="B7" s="4">
+      <c r="B16" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,12,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,1,1))</f>
         <v/>
       </c>
-      <c r="C7" s="4">
+      <c r="C16" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,12,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,1,1))</f>
         <v/>
       </c>
-      <c r="D7" s="4">
+      <c r="D16" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,12,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,1,1))</f>
         <v/>
       </c>
-      <c r="E7" s="4">
+      <c r="E16" s="4">
         <f>SUM(B7:D7)</f>
         <v/>
       </c>
-      <c r="F7" s="4">
+      <c r="F16" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2025,12,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,1,1))</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>01-2026</t>
         </is>
       </c>
-      <c r="B8" s="4">
+      <c r="B17" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,1,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,2,1))</f>
         <v/>
       </c>
-      <c r="C8" s="4">
+      <c r="C17" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,1,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,2,1))</f>
         <v/>
       </c>
-      <c r="D8" s="4">
+      <c r="D17" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,1,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,2,1))</f>
         <v/>
       </c>
-      <c r="E8" s="4">
+      <c r="E17" s="4">
         <f>SUM(B8:D8)</f>
         <v/>
       </c>
-      <c r="F8" s="4">
+      <c r="F17" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,1,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,2,1))</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>02-2026</t>
         </is>
       </c>
-      <c r="B9" s="4">
+      <c r="B18" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,2,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,3,1))</f>
         <v/>
       </c>
-      <c r="C9" s="4">
+      <c r="C18" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,2,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,3,1))</f>
         <v/>
       </c>
-      <c r="D9" s="4">
+      <c r="D18" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,2,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,3,1))</f>
         <v/>
       </c>
-      <c r="E9" s="4">
+      <c r="E18" s="4">
         <f>SUM(B9:D9)</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F18" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,2,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,3,1))</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>03-2026</t>
         </is>
       </c>
-      <c r="B10" s="4">
+      <c r="B19" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,3,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,4,1))</f>
         <v/>
       </c>
-      <c r="C10" s="4">
+      <c r="C19" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,3,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,4,1))</f>
         <v/>
       </c>
-      <c r="D10" s="4">
+      <c r="D19" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,3,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,4,1))</f>
         <v/>
       </c>
-      <c r="E10" s="4">
+      <c r="E19" s="4">
         <f>SUM(B10:D10)</f>
         <v/>
       </c>
-      <c r="F10" s="4">
+      <c r="F19" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,3,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,4,1))</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>04-2026</t>
         </is>
       </c>
-      <c r="B11" s="4">
+      <c r="B20" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,4,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,5,1))</f>
         <v/>
       </c>
-      <c r="C11" s="4">
+      <c r="C20" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,4,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,5,1))</f>
         <v/>
       </c>
-      <c r="D11" s="4">
+      <c r="D20" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,4,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,5,1))</f>
         <v/>
       </c>
-      <c r="E11" s="4">
+      <c r="E20" s="4">
         <f>SUM(B11:D11)</f>
         <v/>
       </c>
-      <c r="F11" s="4">
+      <c r="F20" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,4,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,5,1))</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>05-2026</t>
         </is>
       </c>
-      <c r="B12" s="4">
+      <c r="B21" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,5,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
-      <c r="C12" s="4">
+      <c r="C21" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,5,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
-      <c r="D12" s="4">
+      <c r="D21" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,5,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
-      <c r="E12" s="4">
+      <c r="E21" s="4">
         <f>SUM(B12:D12)</f>
         <v/>
       </c>
-      <c r="F12" s="4">
+      <c r="F21" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,5,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>06-2026</t>
         </is>
       </c>
-      <c r="B13" s="4">
+      <c r="B22" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,6,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
-      <c r="C13" s="4">
+      <c r="C22" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,6,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
-      <c r="D13" s="4">
+      <c r="D22" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,6,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
-      <c r="E13" s="4">
+      <c r="E22" s="4">
         <f>SUM(B13:D13)</f>
         <v/>
       </c>
-      <c r="F13" s="4">
+      <c r="F22" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,6,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>07-2026</t>
         </is>
       </c>
-      <c r="B14" s="4">
+      <c r="B23" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عصمت الله خان",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
-      <c r="C14" s="4">
+      <c r="C23" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"عماد حمدي",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
-      <c r="D14" s="4">
+      <c r="D23" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!C:C,"م/ عادل أبو خالد",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
-      <c r="E14" s="4">
+      <c r="E23" s="4">
         <f>SUM(B14:D14)</f>
         <v/>
       </c>
-      <c r="F14" s="4">
+      <c r="F23" s="4">
         <f>SUMIFS('الحركة المدمجة'!H:H,'الحركة المدمجة'!D:D,"النظام الجديد (السيارات)",'الحركة المدمجة'!B:B,"&gt;="&amp;DATE(2026,7,1),'الحركة المدمجة'!B:B,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B15" s="6">
-        <f>SUM(B2:B14)</f>
+      <c r="B24" s="6">
+        <f>SUM(B2:B23)</f>
         <v/>
       </c>
-      <c r="C15" s="6">
-        <f>SUM(C2:C14)</f>
+      <c r="C24" s="6">
+        <f>SUM(C2:C23)</f>
         <v/>
       </c>
-      <c r="D15" s="6">
-        <f>SUM(D2:D14)</f>
+      <c r="D24" s="6">
+        <f>SUM(D2:D23)</f>
         <v/>
       </c>
-      <c r="E15" s="6">
-        <f>SUM(E2:E14)</f>
+      <c r="E24" s="6">
+        <f>SUM(E2:E23)</f>
         <v/>
       </c>
-      <c r="F15" s="6">
-        <f>SUM(F2:F14)</f>
+      <c r="F24" s="6">
+        <f>SUM(F2:F23)</f>
         <v/>
       </c>
     </row>
@@ -14123,6 +14290,189 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="40" t="inlineStr">
+        <is>
+          <t>مبيعات مزرعة الرياض من 2024-10-01 إلى 2025-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B2" s="39" t="inlineStr">
+        <is>
+          <t>البيان</t>
+        </is>
+      </c>
+      <c r="C2" s="39" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر أكتوبر 2024</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>103500</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر نوفمبر 2024</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>137450</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر ديسمبر 2024</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>95230</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر يناير 2025</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>55300</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر فبراير 2025</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>35920</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر مارس 2025</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>15100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر إبريل 2025</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>90160</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر مايو 2025</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>50310</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات شهر يونيه 2025</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>27718</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>إجمالي المبيعات</t>
+        </is>
+      </c>
+      <c r="C12" s="6">
+        <f>SUM(C3:C11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>ملاحظات: الإجمالي 610,688.00 مطابق لمجموع الأشهر. المبيعات غير موزعة على المناديب. لا توجد بيانات مبيعات للفترة من 1-7-2025 إلى 29-7-2025.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A14:C14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23158,7 +23508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25282,7 +25632,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27033,7 +27383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix shifted row formulas in monthly sales summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/إجمالي_مبيعات_المناديب_30-7-2025_إلى_31-7-2026.xlsx
+++ b/إجمالي_مبيعات_المناديب_30-7-2025_إلى_31-7-2026.xlsx
@@ -13925,7 +13925,7 @@
         <v/>
       </c>
       <c r="E11" s="4">
-        <f>SUM(B2:D2)</f>
+        <f>SUM(B11:D11)</f>
         <v/>
       </c>
       <c r="F11" s="4">
@@ -13952,7 +13952,7 @@
         <v/>
       </c>
       <c r="E12" s="4">
-        <f>SUM(B3:D3)</f>
+        <f>SUM(B12:D12)</f>
         <v/>
       </c>
       <c r="F12" s="4">
@@ -13979,7 +13979,7 @@
         <v/>
       </c>
       <c r="E13" s="4">
-        <f>SUM(B4:D4)</f>
+        <f>SUM(B13:D13)</f>
         <v/>
       </c>
       <c r="F13" s="4">
@@ -14006,7 +14006,7 @@
         <v/>
       </c>
       <c r="E14" s="4">
-        <f>SUM(B5:D5)</f>
+        <f>SUM(B14:D14)</f>
         <v/>
       </c>
       <c r="F14" s="4">
@@ -14033,7 +14033,7 @@
         <v/>
       </c>
       <c r="E15" s="4">
-        <f>SUM(B6:D6)</f>
+        <f>SUM(B15:D15)</f>
         <v/>
       </c>
       <c r="F15" s="4">
@@ -14060,7 +14060,7 @@
         <v/>
       </c>
       <c r="E16" s="4">
-        <f>SUM(B7:D7)</f>
+        <f>SUM(B16:D16)</f>
         <v/>
       </c>
       <c r="F16" s="4">
@@ -14087,7 +14087,7 @@
         <v/>
       </c>
       <c r="E17" s="4">
-        <f>SUM(B8:D8)</f>
+        <f>SUM(B17:D17)</f>
         <v/>
       </c>
       <c r="F17" s="4">
@@ -14114,7 +14114,7 @@
         <v/>
       </c>
       <c r="E18" s="4">
-        <f>SUM(B9:D9)</f>
+        <f>SUM(B18:D18)</f>
         <v/>
       </c>
       <c r="F18" s="4">
@@ -14141,7 +14141,7 @@
         <v/>
       </c>
       <c r="E19" s="4">
-        <f>SUM(B10:D10)</f>
+        <f>SUM(B19:D19)</f>
         <v/>
       </c>
       <c r="F19" s="4">
@@ -14168,7 +14168,7 @@
         <v/>
       </c>
       <c r="E20" s="4">
-        <f>SUM(B11:D11)</f>
+        <f>SUM(B20:D20)</f>
         <v/>
       </c>
       <c r="F20" s="4">
@@ -14195,7 +14195,7 @@
         <v/>
       </c>
       <c r="E21" s="4">
-        <f>SUM(B12:D12)</f>
+        <f>SUM(B21:D21)</f>
         <v/>
       </c>
       <c r="F21" s="4">
@@ -14222,7 +14222,7 @@
         <v/>
       </c>
       <c r="E22" s="4">
-        <f>SUM(B13:D13)</f>
+        <f>SUM(B22:D22)</f>
         <v/>
       </c>
       <c r="F22" s="4">
@@ -14249,7 +14249,7 @@
         <v/>
       </c>
       <c r="E23" s="4">
-        <f>SUM(B14:D14)</f>
+        <f>SUM(B23:D23)</f>
         <v/>
       </c>
       <c r="F23" s="4">

</xml_diff>